<commit_message>
audit log week 3
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example.xlsx
+++ b/AI_AuditLog_Example.xlsx
@@ -59,7 +59,7 @@
     <t>Assignment:</t>
   </si>
   <si>
-    <t>System Booking Travelling</t>
+    <t>Atrraction Booking ticket System</t>
   </si>
   <si>
     <t>AI USAGE SUMMARY</t>
@@ -478,7 +478,7 @@
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -574,13 +574,6 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1066,148 +1059,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>